<commit_message>
update tab error message
</commit_message>
<xml_diff>
--- a/test/data/task_summary.xlsx
+++ b/test/data/task_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,329 +474,6 @@
           <t>Message</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>sbkuzh</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>task_2050-01-01_UZH_LARGE_READY</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2024-08-23 17:23:09</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2050-01-01</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>LARGE</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>sbkrzs</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>task_2034-01-01_RZS_LARGE_ERROR</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2034-01-01</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>LARGE</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Missing file task_2034-01-01_RZS_LARGE.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>sbkrzs</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>task_2033-01-01_RZS_LARGE_ERROR</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2033-01-01</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>LARGE</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Missing file task_2033-01-01_RZS_LARGE.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>sbkzbs</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>task_2033-01-01_ZBS_LARGE_ERROR</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2033-01-01</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>LARGE</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>A large task is already scheduled for this date</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>sbkrzs</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>task_2041-01-01_UBS_LARGE_ERROR</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2041-01-01</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>LARGE</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Missing file task_2041-01-01_UBS_LARGE.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>sbkrzs</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>task_2032-01-01_RZS_LARGE_ERROR</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2032-01-01</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>LARGE</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Missing file task_2032-01-01_RZS_LARGE.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>sbkzbz</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>task_2024-08-25_ZBZ_SMALL_READY</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2024-08-23 17:25:57</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2024-08-25</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>sbkzbz</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>task_2024-08-28_ZBZ3_SMALL_READY</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2024-08-23 17:27:03</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2024-08-28</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>sbkhsg</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>task_2024-08-23_HSG_SMALL_DONE</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2024-08-23 17:27:32</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2024-08-23 17:27:40</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2024-08-23 17:27:52</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2024-08-23</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>SMALL</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>